<commit_message>
made housekeeping changes, added LLM-coverage, updated content
</commit_message>
<xml_diff>
--- a/study_content.xlsx
+++ b/study_content.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\risk-viz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzoc\Desktop\PhD\Other\lorraine\risk-viz\app_content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A560C7-EDCB-4749-B03A-CF19A80319DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5703458-FDAA-4A72-B1C3-30DC236208A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-1245" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="READ ME FIRST" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="237">
   <si>
     <t>How to edit this file</t>
   </si>
@@ -215,9 +215,6 @@
     <t>notice_welcome_body</t>
   </si>
   <si>
-    <t>Up next are examples of flood communication formats and channels. Review and score each one. The SPACE4ALL team will later tailor the project outputs based on your preferences. We will begin shortly 😊</t>
-  </si>
-  <si>
     <t>Body for the welcome-back screen.</t>
   </si>
   <si>
@@ -233,9 +230,6 @@
     <t>notice_completion2_body</t>
   </si>
   <si>
-    <t>We will now move into our last activity of the day, where we will talk about your preferences and identify shared views within the group. Let's go!</t>
-  </si>
-  <si>
     <t>Body for the completion-2 screen.</t>
   </si>
   <si>
@@ -500,69 +494,27 @@
     <t>SMS text alert</t>
   </si>
   <si>
-    <t>images/prompts/sms.png</t>
-  </si>
-  <si>
-    <t>A phone SMS: 'FLOOD ALERT: Heavy rain expected tonight. Move to higher ground if you are near the river.'</t>
-  </si>
-  <si>
     <t>st2</t>
   </si>
   <si>
-    <t>Flood map</t>
-  </si>
-  <si>
-    <t>images/prompts/fd_map.jpg</t>
-  </si>
-  <si>
-    <t>Flood depth map: colour-coded water depth by area.</t>
-  </si>
-  <si>
-    <t>images/prompts/fe_map.jpg</t>
-  </si>
-  <si>
-    <t>Flood extent map: which areas are expected to flood.</t>
-  </si>
-  <si>
     <t>st3</t>
   </si>
   <si>
-    <t>Community radio notice</t>
-  </si>
-  <si>
-    <t>images/prompts/radio.png</t>
-  </si>
-  <si>
-    <t>A spoken radio announcement warning residents of rising water over the next 12 hours.</t>
-  </si>
-  <si>
     <t>wc1</t>
   </si>
   <si>
     <t>wordcloud</t>
   </si>
   <si>
-    <t>Through which channels would you prefer to receive flood information?</t>
-  </si>
-  <si>
     <t>wc2</t>
   </si>
   <si>
-    <t>Which format would be most useful?</t>
-  </si>
-  <si>
     <t>wc3</t>
   </si>
   <si>
-    <t>What is the most important improvement needed in the current flood communication approach you have in place?</t>
-  </si>
-  <si>
     <t>wc4</t>
   </si>
   <si>
-    <t>Is there anything we are missing in today's discussion?</t>
-  </si>
-  <si>
     <t>18-24 years old</t>
   </si>
   <si>
@@ -591,13 +543,205 @@
   </si>
   <si>
     <t>over 10 years</t>
+  </si>
+  <si>
+    <t>What would you like to do with this information?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Through which dissemination channels would you prefer to receive such information? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What type of information would be the best to receive? </t>
+  </si>
+  <si>
+    <t>What would be the most useful format?</t>
+  </si>
+  <si>
+    <t>welcome_title</t>
+  </si>
+  <si>
+    <t>Welcome</t>
+  </si>
+  <si>
+    <t>Title on the first screen participants see.</t>
+  </si>
+  <si>
+    <t>welcome_body</t>
+  </si>
+  <si>
+    <t>Great to have you here! Everything you share is anonymous, so be open and honest. Your insights are essential for shaping flood communication strategies that truly meet your needs. We will begin shortly 😊</t>
+  </si>
+  <si>
+    <t>Body text on the welcome screen (markdown allowed).</t>
+  </si>
+  <si>
+    <t>Up next we will discuss your ideal flood communication approach and identify shared views within the group.. We will begin shortly 😊</t>
+  </si>
+  <si>
+    <t>Flood maps</t>
+  </si>
+  <si>
+    <t>images/prompts/map_01.jpg</t>
+  </si>
+  <si>
+    <t>Flood risk</t>
+  </si>
+  <si>
+    <t>Flood hazard depth</t>
+  </si>
+  <si>
+    <t>st4</t>
+  </si>
+  <si>
+    <t>Evacuation routes map</t>
+  </si>
+  <si>
+    <t>Safe routes</t>
+  </si>
+  <si>
+    <t>images/prompts/evac_01.jpg</t>
+  </si>
+  <si>
+    <t>images/prompts/map_02.png</t>
+  </si>
+  <si>
+    <t>images/prompts/evac_02.png</t>
+  </si>
+  <si>
+    <t>Safe spots map</t>
+  </si>
+  <si>
+    <t>images/prompts/evac_03.png</t>
+  </si>
+  <si>
+    <t>Emergency shelters map</t>
+  </si>
+  <si>
+    <t>Infographic</t>
+  </si>
+  <si>
+    <t>images/prompts/graph_01.png</t>
+  </si>
+  <si>
+    <t>images/prompts/evac_04.png</t>
+  </si>
+  <si>
+    <t>Safe and emergency spots</t>
+  </si>
+  <si>
+    <t>images/prompts/graph_02.jpeg</t>
+  </si>
+  <si>
+    <t>Flood safety</t>
+  </si>
+  <si>
+    <t>Flood prevention</t>
+  </si>
+  <si>
+    <t>images/prompts/graph_03.jpg</t>
+  </si>
+  <si>
+    <t>Flood preparedness</t>
+  </si>
+  <si>
+    <t>Leaflet</t>
+  </si>
+  <si>
+    <t>Banner</t>
+  </si>
+  <si>
+    <t>images/prompts/print_01.gif</t>
+  </si>
+  <si>
+    <t>Notice board</t>
+  </si>
+  <si>
+    <t>images/prompts/print_02.jpg</t>
+  </si>
+  <si>
+    <t>Printed maps</t>
+  </si>
+  <si>
+    <t>images/prompts/print_03.jpg</t>
+  </si>
+  <si>
+    <t>images/prompts/print_04.png</t>
+  </si>
+  <si>
+    <t>st5</t>
+  </si>
+  <si>
+    <t>Radio message</t>
+  </si>
+  <si>
+    <t>images/prompts/radio_01.gif</t>
+  </si>
+  <si>
+    <t>images/prompts/video_01.gif</t>
+  </si>
+  <si>
+    <t>Transmission by radio</t>
+  </si>
+  <si>
+    <t>Transmission by video</t>
+  </si>
+  <si>
+    <t>Transmission by printed means</t>
+  </si>
+  <si>
+    <t>st6</t>
+  </si>
+  <si>
+    <t>st7</t>
+  </si>
+  <si>
+    <t>Transmission by text</t>
+  </si>
+  <si>
+    <t>images/prompts/text_01.jpg</t>
+  </si>
+  <si>
+    <t>images/prompts/text_02.jpg</t>
+  </si>
+  <si>
+    <t>Whatsapp messaging</t>
+  </si>
+  <si>
+    <t>Video via phone</t>
+  </si>
+  <si>
+    <t>Transmission via arts</t>
+  </si>
+  <si>
+    <t>st8</t>
+  </si>
+  <si>
+    <t>images/prompts/arts_01.gif</t>
+  </si>
+  <si>
+    <t>Photo exposition</t>
+  </si>
+  <si>
+    <t>Panel presentation</t>
+  </si>
+  <si>
+    <t>Community theater</t>
+  </si>
+  <si>
+    <t>images/prompts/arts_02.jpeg</t>
+  </si>
+  <si>
+    <t>images/prompts/arts_03.jpg</t>
+  </si>
+  <si>
+    <t>Congratulations! You were amazing today and we greatly appreciate your participation. You can leave the app now and wait for the moderator for final instructions.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,16 +753,25 @@
       <b/>
       <sz val="12"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -634,7 +787,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -657,16 +810,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9DDE2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9DDE2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1188,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1209,112 +1376,134 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="4">
-        <v>5</v>
+        <v>177</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>178</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>43</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>45</v>
+        <v>180</v>
+      </c>
+      <c r="B3" t="s">
+        <v>181</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>46</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
+      </c>
+      <c r="B4" s="4">
+        <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="42" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+    <row r="8" spans="1:3" ht="42" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B8" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="84" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+    <row r="9" spans="1:3" ht="84" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="196" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="126" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="140" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1342,63 +1531,63 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -1406,7 +1595,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1416,7 +1605,7 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1424,7 +1613,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1434,7 +1623,7 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1442,7 +1631,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1452,7 +1641,7 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1460,7 +1649,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1470,7 +1659,7 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1478,25 +1667,25 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1504,7 +1693,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1514,7 +1703,7 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -1522,7 +1711,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1532,7 +1721,7 @@
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
@@ -1540,25 +1729,25 @@
     </row>
     <row r="10" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -1566,7 +1755,7 @@
     </row>
     <row r="11" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1576,7 +1765,7 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -1584,7 +1773,7 @@
     </row>
     <row r="12" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1594,7 +1783,7 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -1602,7 +1791,7 @@
     </row>
     <row r="13" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1612,7 +1801,7 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1620,7 +1809,7 @@
     </row>
     <row r="14" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1630,7 +1819,7 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -1638,25 +1827,25 @@
     </row>
     <row r="15" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -1664,7 +1853,7 @@
     </row>
     <row r="16" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1674,7 +1863,7 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -1682,7 +1871,7 @@
     </row>
     <row r="17" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1692,7 +1881,7 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -1700,7 +1889,7 @@
     </row>
     <row r="18" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1710,7 +1899,7 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
@@ -1718,7 +1907,7 @@
     </row>
     <row r="19" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1728,7 +1917,7 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
@@ -1736,25 +1925,25 @@
     </row>
     <row r="20" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
@@ -1762,7 +1951,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1772,7 +1961,7 @@
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
@@ -1780,7 +1969,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1790,7 +1979,7 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
@@ -1798,7 +1987,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1808,7 +1997,7 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
@@ -1816,7 +2005,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1826,7 +2015,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
@@ -1834,29 +2023,29 @@
     </row>
     <row r="25" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
@@ -1864,7 +2053,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1874,7 +2063,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
@@ -1882,7 +2071,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1892,7 +2081,7 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
@@ -1900,7 +2089,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1910,7 +2099,7 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
@@ -1918,7 +2107,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1928,7 +2117,7 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
@@ -1936,7 +2125,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1946,7 +2135,7 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
@@ -1954,7 +2143,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1964,7 +2153,7 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
@@ -1972,7 +2161,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1982,7 +2171,7 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
@@ -1990,7 +2179,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2000,7 +2189,7 @@
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
@@ -2008,23 +2197,23 @@
     </row>
     <row r="34" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
@@ -2032,7 +2221,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2042,7 +2231,7 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
@@ -2050,7 +2239,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2060,7 +2249,7 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
@@ -2068,7 +2257,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2078,7 +2267,7 @@
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
@@ -2086,23 +2275,23 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -2110,7 +2299,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2120,7 +2309,7 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -2128,7 +2317,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2138,7 +2327,7 @@
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
@@ -2146,7 +2335,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2156,7 +2345,7 @@
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
@@ -2164,25 +2353,25 @@
     </row>
     <row r="42" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
@@ -2190,7 +2379,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2200,7 +2389,7 @@
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J43" s="4"/>
       <c r="K43" s="4"/>
@@ -2208,7 +2397,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -2218,7 +2407,7 @@
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J44" s="4"/>
       <c r="K44" s="4"/>
@@ -2226,7 +2415,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -2236,7 +2425,7 @@
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J45" s="4"/>
       <c r="K45" s="4"/>
@@ -2244,7 +2433,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -2254,7 +2443,7 @@
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J46" s="4"/>
       <c r="K46" s="4"/>
@@ -2262,7 +2451,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -2272,7 +2461,7 @@
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J47" s="4"/>
       <c r="K47" s="4"/>
@@ -2280,7 +2469,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -2290,7 +2479,7 @@
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J48" s="4"/>
       <c r="K48" s="4"/>
@@ -2298,16 +2487,16 @@
     </row>
     <row r="49" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
@@ -2326,16 +2515,16 @@
     </row>
     <row r="50" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
@@ -2352,33 +2541,33 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J51" s="4"/>
       <c r="K51" s="4"/>
       <c r="L51" s="4"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -2388,7 +2577,7 @@
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J52" s="4"/>
       <c r="K52" s="4"/>
@@ -2396,23 +2585,23 @@
     </row>
     <row r="53" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J53" s="4"/>
       <c r="K53" s="4"/>
@@ -2420,7 +2609,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -2430,7 +2619,7 @@
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J54" s="4"/>
       <c r="K54" s="4"/>
@@ -2438,7 +2627,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -2448,7 +2637,7 @@
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
@@ -2456,7 +2645,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -2466,7 +2655,7 @@
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J56" s="4"/>
       <c r="K56" s="4"/>
@@ -2474,16 +2663,16 @@
     </row>
     <row r="57" spans="1:12" ht="28" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
@@ -2507,84 +2696,311 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="2" max="2" width="39.54296875" customWidth="1"/>
+    <col min="3" max="3" width="36.26953125" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="28" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="B2" s="4" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>158</v>
+        <v>185</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="4"/>
+        <v>156</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>190</v>
+      </c>
       <c r="C4" s="4" t="s">
-        <v>164</v>
+        <v>191</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>169</v>
+        <v>194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" t="s">
+        <v>208</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C12" t="s">
+        <v>210</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C14" t="s">
+        <v>213</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="C16" t="s">
+        <v>217</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C17" t="s">
+        <v>224</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C18" t="s">
+        <v>225</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C19" t="s">
+        <v>230</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C20" t="s">
+        <v>234</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C21" t="s">
+        <v>235</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2596,7 +3012,7 @@
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
@@ -2604,36 +3020,36 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>74</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4">
@@ -2648,13 +3064,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -2667,15 +3083,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="42" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4">
@@ -2688,15 +3104,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4">

</xml_diff>

<commit_message>
fixed questionnaire refresh resume, controlled comma/semicolon input in wordcloud, updated LLM-reasoning to semantics not just word frequency
</commit_message>
<xml_diff>
--- a/study_content.xlsx
+++ b/study_content.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzoc\Desktop\PhD\Other\lorraine\risk-viz\app_content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\risk-viz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5703458-FDAA-4A72-B1C3-30DC236208A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89EA6273-0213-474A-98D5-DECDB4D9E198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-1245" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="READ ME FIRST" sheetId="1" r:id="rId1"/>
@@ -371,9 +371,6 @@
     <t>questions</t>
   </si>
   <si>
-    <t>How often have floods affected you or your household?</t>
-  </si>
-  <si>
     <t>Never</t>
   </si>
   <si>
@@ -437,9 +434,6 @@
     <t>word_prompt</t>
   </si>
   <si>
-    <t>Which type of flood-related information do you currently receive?</t>
-  </si>
-  <si>
     <t>info_source</t>
   </si>
   <si>
@@ -735,6 +729,12 @@
   </si>
   <si>
     <t>Congratulations! You were amazing today and we greatly appreciate your participation. You can leave the app now and wait for the moderator for final instructions.</t>
+  </si>
+  <si>
+    <t>How often have you and your household been affected by floods in this community?</t>
+  </si>
+  <si>
+    <t>What type of information do you currently receive regarding floods or extreme weather that leads to floods (storm, tide, opening of dam, etc.)?</t>
   </si>
 </sst>
 </file>
@@ -1139,211 +1139,211 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A42"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>38</v>
       </c>
@@ -1356,14 +1356,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>39</v>
       </c>
@@ -1374,29 +1374,29 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B3" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B3" t="s">
-        <v>181</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>42</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>47</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>50</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="42" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>53</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="84" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>56</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>59</v>
       </c>
@@ -1473,18 +1473,18 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="126" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>64</v>
       </c>
@@ -1495,12 +1495,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="140" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="138" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>67</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>68</v>
@@ -1514,7 +1514,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L57"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1529,7 +1529,7 @@
     <col min="12" max="12" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>69</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>87</v>
       </c>
@@ -1587,13 +1587,13 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>87</v>
       </c>
@@ -1605,13 +1605,13 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>87</v>
       </c>
@@ -1623,13 +1623,13 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>87</v>
       </c>
@@ -1641,13 +1641,13 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>87</v>
       </c>
@@ -1659,13 +1659,13 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>89</v>
       </c>
@@ -1691,7 +1691,7 @@
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>89</v>
       </c>
@@ -1709,7 +1709,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>89</v>
       </c>
@@ -1727,7 +1727,7 @@
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
     </row>
-    <row r="10" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>81</v>
       </c>
@@ -1747,13 +1747,13 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
     </row>
-    <row r="11" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>81</v>
       </c>
@@ -1765,13 +1765,13 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
     </row>
-    <row r="12" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>81</v>
       </c>
@@ -1783,13 +1783,13 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
     </row>
-    <row r="13" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>81</v>
       </c>
@@ -1801,13 +1801,13 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
     </row>
-    <row r="14" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>81</v>
       </c>
@@ -1819,13 +1819,13 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
     </row>
-    <row r="15" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>85</v>
       </c>
@@ -1845,13 +1845,13 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
     </row>
-    <row r="16" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>85</v>
       </c>
@@ -1863,13 +1863,13 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
     </row>
-    <row r="17" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>85</v>
       </c>
@@ -1881,13 +1881,13 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
     </row>
-    <row r="18" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>85</v>
       </c>
@@ -1899,13 +1899,13 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
     </row>
-    <row r="19" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>85</v>
       </c>
@@ -1917,13 +1917,13 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
     </row>
-    <row r="20" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>94</v>
       </c>
@@ -1949,7 +1949,7 @@
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>94</v>
       </c>
@@ -1967,7 +1967,7 @@
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>94</v>
       </c>
@@ -1985,7 +1985,7 @@
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>94</v>
       </c>
@@ -2003,7 +2003,7 @@
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>94</v>
       </c>
@@ -2021,7 +2021,7 @@
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
     </row>
-    <row r="25" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>101</v>
       </c>
@@ -2051,7 +2051,7 @@
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>101</v>
       </c>
@@ -2069,7 +2069,7 @@
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>101</v>
       </c>
@@ -2087,7 +2087,7 @@
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>101</v>
       </c>
@@ -2105,7 +2105,7 @@
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>101</v>
       </c>
@@ -2123,7 +2123,7 @@
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>101</v>
       </c>
@@ -2141,7 +2141,7 @@
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>101</v>
       </c>
@@ -2159,7 +2159,7 @@
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>101</v>
       </c>
@@ -2177,7 +2177,7 @@
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>101</v>
       </c>
@@ -2195,7 +2195,7 @@
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
     </row>
-    <row r="34" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>113</v>
       </c>
@@ -2206,20 +2206,20 @@
         <v>82</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>115</v>
+        <v>235</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>113</v>
       </c>
@@ -2231,13 +2231,13 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>113</v>
       </c>
@@ -2249,13 +2249,13 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>113</v>
       </c>
@@ -2267,15 +2267,15 @@
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>114</v>
@@ -2284,22 +2284,22 @@
         <v>82</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2309,15 +2309,15 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2327,15 +2327,15 @@
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2345,15 +2345,15 @@
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
     </row>
-    <row r="42" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>114</v>
@@ -2362,7 +2362,7 @@
         <v>102</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
@@ -2371,15 +2371,15 @@
         <v>84</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2389,15 +2389,15 @@
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J43" s="4"/>
       <c r="K43" s="4"/>
       <c r="L43" s="4"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -2407,15 +2407,15 @@
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J44" s="4"/>
       <c r="K44" s="4"/>
       <c r="L44" s="4"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -2425,15 +2425,15 @@
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J45" s="4"/>
       <c r="K45" s="4"/>
       <c r="L45" s="4"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -2443,15 +2443,15 @@
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J46" s="4"/>
       <c r="K46" s="4"/>
       <c r="L46" s="4"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -2461,15 +2461,15 @@
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J47" s="4"/>
       <c r="K47" s="4"/>
       <c r="L47" s="4"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -2479,24 +2479,24 @@
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J48" s="4"/>
       <c r="K48" s="4"/>
       <c r="L48" s="4"/>
     </row>
-    <row r="49" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>137</v>
+        <v>236</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
@@ -2504,7 +2504,7 @@
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
       <c r="J49" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K49" s="4">
         <v>1</v>
@@ -2513,18 +2513,18 @@
         <v>30</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
@@ -2532,7 +2532,7 @@
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
       <c r="J50" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K50" s="4">
         <v>1</v>
@@ -2541,9 +2541,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>114</v>
@@ -2552,22 +2552,22 @@
         <v>82</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J51" s="4"/>
       <c r="K51" s="4"/>
       <c r="L51" s="4"/>
     </row>
-    <row r="52" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -2577,39 +2577,39 @@
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J52" s="4"/>
       <c r="K52" s="4"/>
       <c r="L52" s="4"/>
     </row>
-    <row r="53" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J53" s="4"/>
       <c r="K53" s="4"/>
       <c r="L53" s="4"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -2619,15 +2619,15 @@
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J54" s="4"/>
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -2637,15 +2637,15 @@
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
       <c r="L55" s="4"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -2655,24 +2655,24 @@
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J56" s="4"/>
       <c r="K56" s="4"/>
       <c r="L56" s="4"/>
     </row>
-    <row r="57" spans="1:12" ht="28" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
@@ -2680,7 +2680,7 @@
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K57" s="4">
         <v>1</v>
@@ -2697,306 +2697,306 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="39.54296875" customWidth="1"/>
-    <col min="3" max="3" width="36.26953125" customWidth="1"/>
+    <col min="2" max="2" width="39.5546875" customWidth="1"/>
+    <col min="3" max="3" width="36.21875" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>73</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C11" t="s">
+        <v>206</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" t="s">
+        <v>210</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" t="s">
+        <v>211</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C15" t="s">
+        <v>214</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C16" t="s">
+        <v>215</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C17" t="s">
+        <v>222</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="C11" t="s">
-        <v>208</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="C12" t="s">
-        <v>210</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="C13" t="s">
-        <v>212</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="C14" t="s">
-        <v>213</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C15" t="s">
-        <v>216</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="C16" t="s">
-        <v>217</v>
-      </c>
-      <c r="D16" s="5" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="C17" t="s">
-        <v>224</v>
-      </c>
-      <c r="D17" s="5" t="s">
+      <c r="B19" s="5" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="C18" t="s">
-        <v>225</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
+      <c r="C19" t="s">
+        <v>228</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D19" s="5" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C21" t="s">
+        <v>233</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>231</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" t="s">
-        <v>234</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C21" t="s">
-        <v>235</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -3008,17 +3008,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>69</v>
       </c>
@@ -3041,19 +3041,19 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F2" s="4">
         <v>1</v>
@@ -3062,19 +3062,19 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F3" s="4">
         <v>1</v>
@@ -3083,19 +3083,19 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -3104,19 +3104,19 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F5" s="4">
         <v>1</v>

</xml_diff>